<commit_message>
Place tables at top of each sheet, charts below
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Nr1pY8YLdKikwK3qQs9YHw
</commit_message>
<xml_diff>
--- a/reports/주간보고서_2026-10-05_10-09.xlsx
+++ b/reports/주간보고서_2026-10-05_10-09.xlsx
@@ -1696,11 +1696,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="58064962"/>
-        <c:axId val="2610021"/>
+        <c:axId val="15939477"/>
+        <c:axId val="8776893"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="58064962"/>
+        <c:axId val="15939477"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1732,7 +1732,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="2610021"/>
+        <c:crossAx val="8776893"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1740,7 +1740,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="2610021"/>
+        <c:axId val="8776893"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1816,7 +1816,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="58064962"/>
+        <c:crossAx val="15939477"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1998,11 +1998,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="36034870"/>
-        <c:axId val="19480650"/>
+        <c:axId val="14380867"/>
+        <c:axId val="21097323"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="36034870"/>
+        <c:axId val="14380867"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2034,7 +2034,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="19480650"/>
+        <c:crossAx val="21097323"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2042,7 +2042,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="19480650"/>
+        <c:axId val="21097323"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2118,7 +2118,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="36034870"/>
+        <c:crossAx val="14380867"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2373,11 +2373,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="1640733"/>
-        <c:axId val="9472786"/>
+        <c:axId val="18220223"/>
+        <c:axId val="46337484"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="1640733"/>
+        <c:axId val="18220223"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2409,7 +2409,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="9472786"/>
+        <c:crossAx val="46337484"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2417,7 +2417,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="9472786"/>
+        <c:axId val="46337484"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2459,7 +2459,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1640733"/>
+        <c:crossAx val="18220223"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2780,15 +2780,15 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>11</xdr:col>
+      <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>0</xdr:row>
+      <xdr:row>19</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>18</xdr:col>
-      <xdr:colOff>39240</xdr:colOff>
-      <xdr:row>13</xdr:row>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>90360</xdr:colOff>
+      <xdr:row>32</xdr:row>
       <xdr:rowOff>43200</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
@@ -2797,7 +2797,7 @@
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
-        <a:off x="8012520" y="0"/>
+        <a:off x="0" y="3619440"/>
         <a:ext cx="4319640" cy="2519640"/>
       </xdr:xfrm>
       <a:graphic>
@@ -2810,15 +2810,15 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>11</xdr:col>
+      <xdr:col>6</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>15</xdr:row>
+      <xdr:row>19</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>18</xdr:col>
-      <xdr:colOff>39240</xdr:colOff>
-      <xdr:row>28</xdr:row>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>536400</xdr:colOff>
+      <xdr:row>32</xdr:row>
       <xdr:rowOff>43200</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
@@ -2827,7 +2827,7 @@
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
-        <a:off x="8012520" y="2857680"/>
+        <a:off x="4229280" y="3619440"/>
         <a:ext cx="4319640" cy="2519640"/>
       </xdr:xfrm>
       <a:graphic>
@@ -2845,15 +2845,15 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>12</xdr:col>
+      <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>0</xdr:row>
+      <xdr:row>24</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>19</xdr:col>
-      <xdr:colOff>39240</xdr:colOff>
-      <xdr:row>13</xdr:row>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>513360</xdr:colOff>
+      <xdr:row>37</xdr:row>
       <xdr:rowOff>43200</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
@@ -2862,7 +2862,7 @@
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
-        <a:off x="7730640" y="0"/>
+        <a:off x="0" y="4572000"/>
         <a:ext cx="4319640" cy="2519640"/>
       </xdr:xfrm>
       <a:graphic>
@@ -2880,16 +2880,16 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>9</xdr:col>
+      <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>0</xdr:row>
+      <xdr:row>8</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>14</xdr:col>
-      <xdr:colOff>542160</xdr:colOff>
-      <xdr:row>13</xdr:row>
-      <xdr:rowOff>43200</xdr:rowOff>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>75240</xdr:colOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>42840</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -2897,7 +2897,7 @@
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
-        <a:off x="6884640" y="0"/>
+        <a:off x="0" y="1523880"/>
         <a:ext cx="3599640" cy="2519640"/>
       </xdr:xfrm>
       <a:graphic>

</xml_diff>

<commit_message>
Regenerate weekly report from source files (totals verified)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Nr1pY8YLdKikwK3qQs9YHw
</commit_message>
<xml_diff>
--- a/reports/주간보고서_2026-10-05_10-09.xlsx
+++ b/reports/주간보고서_2026-10-05_10-09.xlsx
@@ -1696,11 +1696,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="15939477"/>
-        <c:axId val="8776893"/>
+        <c:axId val="86281437"/>
+        <c:axId val="72424502"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="15939477"/>
+        <c:axId val="86281437"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1732,7 +1732,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="8776893"/>
+        <c:crossAx val="72424502"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1740,7 +1740,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="8776893"/>
+        <c:axId val="72424502"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1816,7 +1816,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="15939477"/>
+        <c:crossAx val="86281437"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1998,11 +1998,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="14380867"/>
-        <c:axId val="21097323"/>
+        <c:axId val="75818002"/>
+        <c:axId val="55735773"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="14380867"/>
+        <c:axId val="75818002"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2034,7 +2034,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="21097323"/>
+        <c:crossAx val="55735773"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2042,7 +2042,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="21097323"/>
+        <c:axId val="55735773"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2118,7 +2118,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="14380867"/>
+        <c:crossAx val="75818002"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2373,11 +2373,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="18220223"/>
-        <c:axId val="46337484"/>
+        <c:axId val="5011355"/>
+        <c:axId val="64798799"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="18220223"/>
+        <c:axId val="5011355"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2409,7 +2409,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="46337484"/>
+        <c:crossAx val="64798799"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2417,7 +2417,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="46337484"/>
+        <c:axId val="64798799"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2459,7 +2459,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="18220223"/>
+        <c:crossAx val="5011355"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>

</xml_diff>